<commit_message>
DEC-003 v0.5 and Decision Log v0.10: RC evidence filled in (DEC-006, DEC-012, DEC-015, DEC-017), CR approvals of 17/10 (DEC-005, DEC-016, DEC-017), M4 contention and RSK-019 trigger (DEC-010, DEC-016); DEC-003 matches #133 as merged (NODE_ENV, proxy_http_version, live files kept for IPv6)
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.10.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\decisions\Decision Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9280C0FC-2458-4544-B8D8-AA0BA5C83547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52015865-4650-4EFE-AFFC-193E53F9D2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -407,9 +407,6 @@
     <t>Playwright pinned at @playwright/test 1.64.0 (exact, e2e/package.json; Chromium build 1248). Recorded local E2E run: docs/evidence/M3-e2e/E2E_local_run_2026-10-12.txt (12/10/2026, 21:27 UTC, test cluster, exit code 0): E2E-1 and E2E-2a pass, E2E-2b an expected failure with its 422 quoted. Still required: the client build step in DEC-003 before the staging run.</t>
   </si>
   <si>
-    <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. Cells marked [Sunday RC check] are completed from the v4.0-M4-rc evidence before this version merges.</t>
-  </si>
-  <si>
     <t>Final status (M4)</t>
   </si>
   <si>
@@ -443,15 +440,6 @@
     <t>Held as a team position; never validated by STK-009</t>
   </si>
   <si>
-    <t>The one-month period stands, but it was never confirmed with the information officer (OI-12 stays open). It is enforced only by running PROC-001 by hand (scripts/retention/proc-001-anonymise.js); automated enforcement (SCP-020) stayed deferred. Its conflict with FR-6.7 is carried as OI-13 / CR-003.</t>
-  </si>
-  <si>
-    <t>Held [Sunday RC check]</t>
-  </si>
-  <si>
-    <t>Request submission was not built through M3, so the decision was not exercised until M4. [Sunday RC check: whether the M4 submission form requires exactly category, location and description, with the v4.0-M4-rc evidence.]</t>
-  </si>
-  <si>
     <t>Superseded by DEC-013 (unchanged)</t>
   </si>
   <si>
@@ -467,45 +455,18 @@
     <t>Not put into operation; NFR-1.5 not evidenced</t>
   </si>
   <si>
-    <t>The backup and restore scripts exist (scripts/backup/), but the institutional server (E1) was never confirmed, so no dump or restore test has run in any environment. The free tier held under the M3 load: NFR-2.4 passed on staging at 11.04 requests/s. The 70 % of 100 ops/s trigger was not measured (RSK-019). Real production use is one of its own re-open conditions, so it must be re-decided before production.</t>
-  </si>
-  <si>
     <t>Held in code; subscribers not registered</t>
   </si>
   <si>
     <t>The transition service publishes after commit, and the history entry is written inside the transaction, not by a subscriber. The two subscribers, requester feedback and reportingCounts, are not registered (TD-001). Publish therefore has no listeners, and the reporting projection has no recovery path (OI-14). The extensibility benefit was never exercised: SCP-014 was not admitted.</t>
   </si>
   <si>
-    <t>Partly built: points 1 and 2; point 3 not built [Sunday RC check]</t>
-  </si>
-  <si>
-    <t>The route guard (point 1) and the object-level checks (point 2) are built and tested, and an unguarded route fails CI. Point 3, the field-level serialiser, was not built because CFL-002 / OI-16 was never confirmed with STK-006. In its place, the whole read of a security-category request is refused to staff who are not Security Officers, which is stricter than FR-1.5 (OI-17). [Sunday RC check: confirm that this is unchanged at v4.0-M4-rc.]</t>
-  </si>
-  <si>
     <t>The client is responsive web only. Browser coverage (NFR-1.1) is not claimed: E2E runs on Chromium only (DEC-019), and the BC browser set was never confirmed (OI-07).</t>
   </si>
   <si>
     <t>The layer rule is enforced: CI fails a merge when a route or middleware file imports a model or repository, as GATE-01 showed (run 38357191208, 13/10/2026). The check covers src/routes and src/middleware only. One application instance remains a single point of failure (RSK-017).</t>
   </si>
   <si>
-    <t>Held; five differences found by tests [Sunday RC check]</t>
-  </si>
-  <si>
-    <t>The integration cases were written to DEC-015 before the code and found five differences inherited from the M2 slice: DEF-007 to DEF-011, 15 of 40 checks failing at M3. The same 15 fail in CI on a throwaway replica set (PR #122). The client sends a fresh key for every transition, so DEF-009 does not reach it. [Sunday RC check: record which differences the M4 fixes closed, with the CI integration result at v4.0-M4-rc.]</t>
-  </si>
-  <si>
-    <t>Held; verified</t>
-  </si>
-  <si>
-    <t>The transaction-boundary case passes: a failure after both writes and before commit persists neither and publishes nothing, on the test cluster at M3 and in CI (PR #122). The unique index behind its concurrency rule, (requestId, requestVersion), was absent on the test cluster until TD-004's provisioning closed DEF-015 (14 and 15/10/2026). CR-001 (AC-NFR-1.10 v0.3) is still Proposed.</t>
-  </si>
-  <si>
-    <t>Held; enforcement manual</t>
-  </si>
-  <si>
-    <t>Retention per purpose stands, and OI-06 stays closed. Purpose A is enforced only by running PROC-001 by hand; SCP-020 stays deferred. The FR-6.7 conflict it exposed is OI-13 / CR-003. [Sunday RC check: CR-003's final status as PED v4.0 records it.]</t>
-  </si>
-  <si>
     <t>Held; login throttling deliberately absent</t>
   </si>
   <si>
@@ -513,6 +474,45 @@
   </si>
   <si>
     <t>The Vite build and Playwright E2E were used as decided. At the M3 tag E2E-1 and E2E-2a pass, and E2E-2b is an expected failure on DEF-011. It exposed the missing client build step in DEC-003, which was added at v0.3. On staging the client was then built but not served until 15/10/2026 (DEF-021). E2E does not run in CI, and it was not run on staging at M3.</t>
+  </si>
+  <si>
+    <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. The cells that waited on the release candidate (DEC-006, DEC-012, DEC-015, DEC-017) were completed on 18/10/2026 from the v4.0-M4-rc evidence, and the DEC-005, DEC-010, DEC-016 and DEC-017 consequences were brought up to date with the CR approvals of 17/10/2026 and the staging runs of 18/10/2026.</t>
+  </si>
+  <si>
+    <t>The one-month period stands, but it was never confirmed with the information officer (OI-12 stays open). It is enforced only by running PROC-001 by hand (scripts/retention/proc-001-anonymise.js); automated enforcement (SCP-020) stayed deferred. Its conflict with FR-6.7 was settled by CR-003, approved by the team on 17/10/2026 (not validated with a client stakeholder), which closes OI-13.</t>
+  </si>
+  <si>
+    <t>Held; exercised at M4 and met</t>
+  </si>
+  <si>
+    <t>Request submission was not built through M3, so the decision was not exercised until M4. At M4 the submission form and API require exactly category, location and description: AC-FR-2.2a and AC-FR-2.2b are Met at the frozen build 6408ab7 (E2E-3; a missing field returns 400 and nothing is stored; RTM v0.11).</t>
+  </si>
+  <si>
+    <t>The backup and restore scripts exist (scripts/backup/), but the institutional server (E1) was never confirmed, so no dump or restore test has run in any environment. The free tier held under the M3 load: NFR-2.4 passed on staging at 11.04 requests/s. The 70 % of 100 ops/s trigger was not measured (RSK-019). Real production use is one of its own re-open conditions, so it must be re-decided before production. M4 (18/10/2026): the trigger was reached. The NFR-2.4 run on staging at v4.0-M4-rc took Atlas to about 74 ops/s, over 70 % of 100 ops/s, so DEC-010's own re-open condition is met (M4 staging deploy record).</t>
+  </si>
+  <si>
+    <t>Partly built: points 1 and 2; point 3 not built at v4.0-M4-rc</t>
+  </si>
+  <si>
+    <t>The route guard (point 1) and the object-level checks (point 2) are built and tested, and an unguarded route fails CI. Point 3, the field-level serialiser, was not built because CFL-002 / OI-16 was never confirmed with STK-006. In its place, the whole read of a security-category request is refused to staff who are not Security Officers, which is stricter than FR-1.5 (OI-17). Unchanged at v4.0-M4-rc: AC-FR-1.5 is Partially Met (RTM v0.11). DEF-024 (S1: a per-viewer response reused from the browser cache after a user switch) was this risk materialising in the client; it was fixed with Cache-Control: no-store and is covered by E2E-10.</t>
+  </si>
+  <si>
+    <t>Held; the five differences fixed at M4 (DEF-007 to DEF-011)</t>
+  </si>
+  <si>
+    <t>The integration cases were written to DEC-015 before the code and found five differences inherited from the M2 slice: DEF-007 to DEF-011, 15 of 40 checks failing at M3. The same 15 fail in CI on a throwaway replica set (PR #122). The client sends a fresh key for every transition, so DEF-009 does not reach it. All five were fixed in PR #136 (804138f, e973a9d): the integration cases pass 40 of 40 at the frozen build 6408ab7 and in CI on dev (run 39079571516). The routes DEC-015 v0.1 did not list were settled before they were built (DEC-015 Addendum A, 17/10/2026). E2E passed 56 of 56 in four browsers at 6408ab7, and the four-role walkthrough on staging at v4.0-M4-rc (CC-2026-000521, 18/10/2026) matched every step.</t>
+  </si>
+  <si>
+    <t>Held; verified; submission contention found at M4</t>
+  </si>
+  <si>
+    <t>The transaction-boundary case passes: a failure after both writes and before commit persists neither and publishes nothing, on the test cluster at M3 and in CI (PR #122). The unique index behind its concurrency rule, (requestId, requestVersion), was absent on the test cluster until TD-004's provisioning closed DEF-015 (14 and 15/10/2026). CR-001 (AC-NFR-1.10 v0.3) was approved by the team on 17/10/2026 (not validated with a client stakeholder). M4 consequence: the FR-2.6 sequential reference is taken by incrementing one counter document inside the same create transaction (counterRepository.js, unitOfWork.js). Under 100 simultaneous submissions on staging (NFR-2.1, 18/10/2026) the transactions write-conflicted on that document (WriteConflict, code 112), and the driver re-ran them for up to 120 s. 30 of 100 were not saved, and 43 were saved after the client had gone. NFR-2.4 failed the same way (17 of 450 submissions timed out at the client, all saved). The proposed fix takes the number with an atomic $inc before the transaction (FR-2.6 needs unique and immutable, not gap-free).</t>
+  </si>
+  <si>
+    <t>Held; enforcement manual; CR-003 approved</t>
+  </si>
+  <si>
+    <t>Retention per purpose stands, and OI-06 stays closed. Purpose A is enforced only by running PROC-001 by hand; SCP-020 stays deferred. The FR-6.7 conflict it exposed (OI-13) was settled by CR-003, approved by the team on 17/10/2026 and not validated with a client stakeholder. Functional Requirements v0.3 holds the FR-6.7 basis, and OI-13 is closed (Open Items v0.8).</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="28" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
@@ -1251,10 +1251,10 @@
         <v>10</v>
       </c>
       <c r="L4" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="N4" s="24" t="s">
         <v>11</v>
@@ -1295,10 +1295,10 @@
         <v>19</v>
       </c>
       <c r="L5" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="M5" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="N5" s="27" t="s">
         <v>20</v>
@@ -1342,10 +1342,10 @@
         <v>19</v>
       </c>
       <c r="L6" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="M6" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="N6" s="27" t="s">
         <v>27</v>
@@ -1389,10 +1389,10 @@
         <v>19</v>
       </c>
       <c r="L7" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>132</v>
       </c>
       <c r="N7" s="26" t="s">
         <v>34</v>
@@ -1436,10 +1436,10 @@
         <v>19</v>
       </c>
       <c r="L8" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="M8" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>134</v>
       </c>
       <c r="N8" s="20" t="s">
         <v>40</v>
@@ -1483,10 +1483,10 @@
         <v>19</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1522,10 +1522,10 @@
         <v>19</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="2:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1561,10 +1561,10 @@
         <v>57</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1600,10 +1600,10 @@
         <v>19</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="2:16" ht="160.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1639,10 +1639,10 @@
         <v>19</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="2:16" ht="150" customHeight="1" x14ac:dyDescent="0.25">
@@ -1678,10 +1678,10 @@
         <v>19</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="M14" s="17" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" spans="2:16" ht="299.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1717,10 +1717,10 @@
         <v>20</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="2:16" ht="360" customHeight="1" x14ac:dyDescent="0.25">
@@ -1756,10 +1756,10 @@
         <v>20</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1795,10 +1795,10 @@
         <v>19</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1834,10 +1834,10 @@
         <v>19</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1873,10 +1873,10 @@
         <v>19</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1912,10 +1912,10 @@
         <v>19</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1951,10 +1951,10 @@
         <v>19</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1990,10 +1990,10 @@
         <v>19</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="2:13" ht="268.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -2029,10 +2029,10 @@
         <v>19</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DEC-003 v0.5: staging domain civicconnect.co.za with a Let's Encrypt certificate since 18/10/2026 (Edge row, step 7, Staging row, change note); Decision Log v0.10: DEC-016 cites DEF-032 and the undeployed audit trigger, DEC-003 domain note, DEC-015 integration job required
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.10.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\decisions\Decision Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52015865-4650-4EFE-AFFC-193E53F9D2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3A6926-FE0C-4ED3-AE37-1B0D1FD3936E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -428,9 +428,6 @@
     <t>Revised (DEC-003 v0.5): staging decided and built; production host undecided</t>
   </si>
   <si>
-    <t>v0.1 to v0.3 rested on a VPS that never existed (OI-21), found only when someone was asked to deploy, and staging moved to a disposable Azure VM (v0.4). The first staging deploy (15/10/2026) found two configuration faults that the health check could not see: a URI without the database name (DEF-020) and the client not served (DEF-021). v0.5 does four things. It records the hand deploy. It moves the Nginx and systemd files into the repository (PR #133). It accepts non-colocation and the self-signed certificate for staging. It leaves production without a host, so no production release is possible under it.</t>
-  </si>
-  <si>
     <t>Held</t>
   </si>
   <si>
@@ -476,9 +473,6 @@
     <t>The Vite build and Playwright E2E were used as decided. At the M3 tag E2E-1 and E2E-2a pass, and E2E-2b is an expected failure on DEF-011. It exposed the missing client build step in DEC-003, which was added at v0.3. On staging the client was then built but not served until 15/10/2026 (DEF-021). E2E does not run in CI, and it was not run on staging at M3.</t>
   </si>
   <si>
-    <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. The cells that waited on the release candidate (DEC-006, DEC-012, DEC-015, DEC-017) were completed on 18/10/2026 from the v4.0-M4-rc evidence, and the DEC-005, DEC-010, DEC-016 and DEC-017 consequences were brought up to date with the CR approvals of 17/10/2026 and the staging runs of 18/10/2026.</t>
-  </si>
-  <si>
     <t>The one-month period stands, but it was never confirmed with the information officer (OI-12 stays open). It is enforced only by running PROC-001 by hand (scripts/retention/proc-001-anonymise.js); automated enforcement (SCP-020) stayed deferred. Its conflict with FR-6.7 was settled by CR-003, approved by the team on 17/10/2026 (not validated with a client stakeholder), which closes OI-13.</t>
   </si>
   <si>
@@ -500,19 +494,25 @@
     <t>Held; the five differences fixed at M4 (DEF-007 to DEF-011)</t>
   </si>
   <si>
-    <t>The integration cases were written to DEC-015 before the code and found five differences inherited from the M2 slice: DEF-007 to DEF-011, 15 of 40 checks failing at M3. The same 15 fail in CI on a throwaway replica set (PR #122). The client sends a fresh key for every transition, so DEF-009 does not reach it. All five were fixed in PR #136 (804138f, e973a9d): the integration cases pass 40 of 40 at the frozen build 6408ab7 and in CI on dev (run 39079571516). The routes DEC-015 v0.1 did not list were settled before they were built (DEC-015 Addendum A, 17/10/2026). E2E passed 56 of 56 in four browsers at 6408ab7, and the four-role walkthrough on staging at v4.0-M4-rc (CC-2026-000521, 18/10/2026) matched every step.</t>
-  </si>
-  <si>
     <t>Held; verified; submission contention found at M4</t>
   </si>
   <si>
-    <t>The transaction-boundary case passes: a failure after both writes and before commit persists neither and publishes nothing, on the test cluster at M3 and in CI (PR #122). The unique index behind its concurrency rule, (requestId, requestVersion), was absent on the test cluster until TD-004's provisioning closed DEF-015 (14 and 15/10/2026). CR-001 (AC-NFR-1.10 v0.3) was approved by the team on 17/10/2026 (not validated with a client stakeholder). M4 consequence: the FR-2.6 sequential reference is taken by incrementing one counter document inside the same create transaction (counterRepository.js, unitOfWork.js). Under 100 simultaneous submissions on staging (NFR-2.1, 18/10/2026) the transactions write-conflicted on that document (WriteConflict, code 112), and the driver re-ran them for up to 120 s. 30 of 100 were not saved, and 43 were saved after the client had gone. NFR-2.4 failed the same way (17 of 450 submissions timed out at the client, all saved). The proposed fix takes the number with an atomic $inc before the transaction (FR-2.6 needs unique and immutable, not gap-free).</t>
-  </si>
-  <si>
     <t>Held; enforcement manual; CR-003 approved</t>
   </si>
   <si>
     <t>Retention per purpose stands, and OI-06 stays closed. Purpose A is enforced only by running PROC-001 by hand; SCP-020 stays deferred. The FR-6.7 conflict it exposed (OI-13) was settled by CR-003, approved by the team on 17/10/2026 and not validated with a client stakeholder. Functional Requirements v0.3 holds the FR-6.7 basis, and OI-13 is closed (Open Items v0.8).</t>
+  </si>
+  <si>
+    <t>The transaction-boundary case passes: a failure after both writes and before commit persists neither and publishes nothing, on the test cluster at M3 and in CI (PR #122). The unique index behind its concurrency rule, (requestId, requestVersion), was absent on the test cluster until TD-004's provisioning closed DEF-015 (14 and 15/10/2026). CR-001 (AC-NFR-1.10 v0.3) was approved by the team on 17/10/2026 (not validated with a client stakeholder). The case shows the clauses that do not depend on the Atlas trigger; the trigger is not deployed, so the two auditLog clauses are not shown. M4 consequence: the FR-2.6 sequential reference is taken by incrementing one counter document inside the same create transaction (counterRepository.js, unitOfWork.js). Under 100 simultaneous submissions on staging (NFR-2.1, 18/10/2026) the transactions write-conflicted on that document (WriteConflict, code 112), and the driver re-ran them for up to 120 s. 30 of 100 were not saved, and 43 were saved after the client had gone. NFR-2.4 failed the same way (17 of 450 submissions timed out at the client, all saved). The proposed fix takes the number with an atomic $inc before the transaction (FR-2.6 needs unique and immutable, not gap-free). Recorded as DEF-032 (S1, P2).</t>
+  </si>
+  <si>
+    <t>v0.1 to v0.3 rested on a VPS that never existed (OI-21), found only when someone was asked to deploy, and staging moved to a disposable Azure VM (v0.4). The first staging deploy (15/10/2026) found two configuration faults that the health check could not see: a URI without the database name (DEF-020) and the client not served (DEF-021). v0.5 does four things. It records the hand deploy. It moves the Nginx and systemd files into the repository (PR #133). It accepts non-colocation and the self-signed certificate for staging. It leaves production without a host, so no production release is possible under it. Since 18/10/2026 12:15 UTC staging serves https://civicconnect.co.za with a Let's Encrypt certificate; the release-candidate checks ran on the self-signed certificate before it (DEC-003 v0.5, Edge row).</t>
+  </si>
+  <si>
+    <t>The integration cases were written to DEC-015 before the code and found five differences inherited from the M2 slice: DEF-007 to DEF-011, 15 of 40 checks failing at M3. The same 15 fail in CI on a throwaway replica set (PR #122). The client sends a fresh key for every transition, so DEF-009 does not reach it. All five were fixed in PR #136 (804138f, e973a9d): the integration cases pass 40 of 40 at the frozen build 6408ab7 and in CI on dev (run 39079571516). The routes DEC-015 v0.1 did not list were settled before they were built (DEC-015 Addendum A, 17/10/2026). E2E passed 56 of 56 in four browsers at 6408ab7, and the four-role walkthrough on staging at v4.0-M4-rc (CC-2026-000521, 18/10/2026) matched every step. The CI integration job has been a required check on dev since 18/10/2026 (TD-008 repaid).</t>
+  </si>
+  <si>
+    <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. The cells that waited on the release candidate (DEC-006, DEC-012, DEC-015, DEC-017) were completed on 18/10/2026 from the v4.0-M4-rc evidence, and the DEC-005, DEC-010, DEC-016 and DEC-017 consequences were brought up to date with the CR approvals of 17/10/2026 and the staging runs of 18/10/2026. DEC-016 cites DEF-032; DEC-003 records the staging domain and certificate of 18/10/2026; DEC-015 records the integration job as a required check.</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="28" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
@@ -1392,7 +1392,7 @@
         <v>130</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="N7" s="26" t="s">
         <v>34</v>
@@ -1436,10 +1436,10 @@
         <v>19</v>
       </c>
       <c r="L8" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="M8" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="N8" s="20" t="s">
         <v>40</v>
@@ -1483,10 +1483,10 @@
         <v>19</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1522,10 +1522,10 @@
         <v>19</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="2:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1561,10 +1561,10 @@
         <v>57</v>
       </c>
       <c r="L11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="M11" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1600,10 +1600,10 @@
         <v>19</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="2:16" ht="160.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1639,10 +1639,10 @@
         <v>19</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="2:16" ht="150" customHeight="1" x14ac:dyDescent="0.25">
@@ -1678,10 +1678,10 @@
         <v>19</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="M14" s="17" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="2:16" ht="299.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1717,10 +1717,10 @@
         <v>20</v>
       </c>
       <c r="L15" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="M15" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="16" spans="2:16" ht="360" customHeight="1" x14ac:dyDescent="0.25">
@@ -1756,10 +1756,10 @@
         <v>20</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1795,10 +1795,10 @@
         <v>19</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1834,10 +1834,10 @@
         <v>19</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1873,10 +1873,10 @@
         <v>19</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1912,10 +1912,10 @@
         <v>19</v>
       </c>
       <c r="L20" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="M20" s="10" t="s">
         <v>156</v>
-      </c>
-      <c r="M20" s="10" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="21" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1951,10 +1951,10 @@
         <v>19</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="22" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1990,10 +1990,10 @@
         <v>19</v>
       </c>
       <c r="L22" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="M22" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="M22" s="10" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="23" spans="2:13" ht="268.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -2029,10 +2029,10 @@
         <v>19</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Decision Log v0.10 review fixes: DEC-011 notification subscriber registered (L15, M15); DEC-004 DEF-011 fixed, DEC-013 and DEC-019 four-browser E2E at M4, DEC-018 login p50 at M3 and M4 (M8, M17, M22, M23); DEC-003 v0.5 change note on the staging domain
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.10.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\decisions\Decision Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3A6926-FE0C-4ED3-AE37-1B0D1FD3936E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EAE6CE6-3AEF-4A84-B50F-33F6FB151391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -431,9 +431,6 @@
     <t>Held</t>
   </si>
   <si>
-    <t>Authorisation was designed in, not retrofitted. The route guard is composed once, and a route-table test fails the build if a non-public route lacks it (NFR-3.3). The integration tests caught the wrong-role status (DEF-011). The field-level part, DEC-012 point 3, was not built (OI-16).</t>
-  </si>
-  <si>
     <t>Held as a team position; never validated by STK-009</t>
   </si>
   <si>
@@ -452,27 +449,12 @@
     <t>Not put into operation; NFR-1.5 not evidenced</t>
   </si>
   <si>
-    <t>Held in code; subscribers not registered</t>
-  </si>
-  <si>
-    <t>The transition service publishes after commit, and the history entry is written inside the transaction, not by a subscriber. The two subscribers, requester feedback and reportingCounts, are not registered (TD-001). Publish therefore has no listeners, and the reporting projection has no recovery path (OI-14). The extensibility benefit was never exercised: SCP-014 was not admitted.</t>
-  </si>
-  <si>
-    <t>The client is responsive web only. Browser coverage (NFR-1.1) is not claimed: E2E runs on Chromium only (DEC-019), and the BC browser set was never confirmed (OI-07).</t>
-  </si>
-  <si>
     <t>The layer rule is enforced: CI fails a merge when a route or middleware file imports a model or repository, as GATE-01 showed (run 38357191208, 13/10/2026). The check covers src/routes and src/middleware only. One application instance remains a single point of failure (RSK-017).</t>
   </si>
   <si>
     <t>Held; login throttling deliberately absent</t>
   </si>
   <si>
-    <t>Local accounts, scrypt hashing and server-side sessions are built and tested. A test asserts the session cookie's security attributes; it failed intermittently twice, cause unknown (DEF-013). Login has no throttling: CodeQL alert #1 (missing rate limiting) has been open since PR #83, and RSK-021 is accepted, not mitigated. This blocks production use. Under the NFR-2.4 load on staging, login took 430 ms at p50, including the South Africa to Spain round trip.</t>
-  </si>
-  <si>
-    <t>The Vite build and Playwright E2E were used as decided. At the M3 tag E2E-1 and E2E-2a pass, and E2E-2b is an expected failure on DEF-011. It exposed the missing client build step in DEC-003, which was added at v0.3. On staging the client was then built but not served until 15/10/2026 (DEF-021). E2E does not run in CI, and it was not run on staging at M3.</t>
-  </si>
-  <si>
     <t>The one-month period stands, but it was never confirmed with the information officer (OI-12 stays open). It is enforced only by running PROC-001 by hand (scripts/retention/proc-001-anonymise.js); automated enforcement (SCP-020) stayed deferred. Its conflict with FR-6.7 was settled by CR-003, approved by the team on 17/10/2026 (not validated with a client stakeholder), which closes OI-13.</t>
   </si>
   <si>
@@ -512,7 +494,25 @@
     <t>The integration cases were written to DEC-015 before the code and found five differences inherited from the M2 slice: DEF-007 to DEF-011, 15 of 40 checks failing at M3. The same 15 fail in CI on a throwaway replica set (PR #122). The client sends a fresh key for every transition, so DEF-009 does not reach it. All five were fixed in PR #136 (804138f, e973a9d): the integration cases pass 40 of 40 at the frozen build 6408ab7 and in CI on dev (run 39079571516). The routes DEC-015 v0.1 did not list were settled before they were built (DEC-015 Addendum A, 17/10/2026). E2E passed 56 of 56 in four browsers at 6408ab7, and the four-role walkthrough on staging at v4.0-M4-rc (CC-2026-000521, 18/10/2026) matched every step. The CI integration job has been a required check on dev since 18/10/2026 (TD-008 repaid).</t>
   </si>
   <si>
-    <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. The cells that waited on the release candidate (DEC-006, DEC-012, DEC-015, DEC-017) were completed on 18/10/2026 from the v4.0-M4-rc evidence, and the DEC-005, DEC-010, DEC-016 and DEC-017 consequences were brought up to date with the CR approvals of 17/10/2026 and the staging runs of 18/10/2026. DEC-016 cites DEF-032; DEC-003 records the staging domain and certificate of 18/10/2026; DEC-015 records the integration job as a required check.</t>
+    <t>Held; the notification subscriber is registered, the reportingCounts projection is not (TD-001 partly repaid)</t>
+  </si>
+  <si>
+    <t>The transition service publishes after commit, and the history entry is written inside the transaction, not by a subscriber. At M4 the notification subscriber is registered (src/composition.js, registerSubscribers), so each status change creates an in-application notification for the requester (FR-3.4, Met at the frozen build 6408ab7). The reportingCounts projection is not registered (TD-001 partly repaid): the management view built at M4 counts from requests directly (FR-8.1 to FR-8.6 Met), so the projection and its recovery path (OI-14) are unused. SCP-014 was not admitted.</t>
+  </si>
+  <si>
+    <t>Authorisation was designed in, not retrofitted. The route guard is composed once, and a route-table test fails the build if a non-public route lacks it (NFR-3.3). The integration tests caught the wrong-role status (DEF-011), which was fixed in PR #136: a role not permitted for a transition now gets 403 (integration 40 of 40 at 6408ab7). The field-level part, DEC-012 point 3, was not built (OI-16).</t>
+  </si>
+  <si>
+    <t>The client is responsive web only. Browser coverage (NFR-1.1) is Partially Met: at M4 the E2E journeys ran 56 of 56 in four browser projects (Chromium, Chrome, Edge and Playwright's Firefox) at 6408ab7, but prior browser releases and Mozilla's release Firefox are not shown (RTM v0.11), and the BC browser set was never confirmed (OI-07).</t>
+  </si>
+  <si>
+    <t>Local accounts, scrypt hashing and server-side sessions are built and tested. A test asserts the session cookie's security attributes; it failed intermittently twice, cause unknown (DEF-013). Login has no throttling: CodeQL alert #1 (missing rate limiting) has been open since PR #83, and RSK-021 is accepted, not mitigated. This blocks production use. Under the NFR-2.4 load on staging, login took 430 ms at p50 at M3 (15/10/2026) and 432 ms at M4 (v4.0-M4-rc, 18/10/2026), including the South Africa to Spain round trip.</t>
+  </si>
+  <si>
+    <t>The Vite build and Playwright E2E were used as decided. At the M3 tag E2E-1 and E2E-2a pass, and E2E-2b is an expected failure on DEF-011. It exposed the missing client build step in DEC-003, which was added at v0.3. On staging the client was then built but not served until 15/10/2026 (DEF-021). It was not run on staging at M3. At M4, DEF-011 was fixed and E2E-2b's expected-failure mark removed (PR #136), and E2E ran 56 of 56 in four browsers at 6408ab7. E2E still does not run in CI.</t>
+  </si>
+  <si>
+    <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. The cells that waited on the release candidate (DEC-006, DEC-012, DEC-015, DEC-017) were completed on 18/10/2026 from the v4.0-M4-rc evidence, and the DEC-005, DEC-010, DEC-016 and DEC-017 consequences were brought up to date with the CR approvals of 17/10/2026 and the staging runs of 18/10/2026. DEC-016 cites DEF-032; DEC-003 records the staging domain and certificate of 18/10/2026; DEC-015 records the integration job as a required check. After review (18/10/2026): DEC-011 (L15, M15) records the registered notification subscriber, and DEC-004, DEC-013, DEC-018 and DEC-019 (M8, M17, M22, M23) record the M4 fixes and four-browser E2E runs.</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1392,7 @@
         <v>130</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="N7" s="26" t="s">
         <v>34</v>
@@ -1439,7 +1439,7 @@
         <v>131</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="N8" s="20" t="s">
         <v>40</v>
@@ -1483,10 +1483,10 @@
         <v>19</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1522,10 +1522,10 @@
         <v>19</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="2:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1561,10 +1561,10 @@
         <v>57</v>
       </c>
       <c r="L11" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="M11" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1603,7 +1603,7 @@
         <v>131</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="2:16" ht="160.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1642,7 +1642,7 @@
         <v>131</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="2:16" ht="150" customHeight="1" x14ac:dyDescent="0.25">
@@ -1678,10 +1678,10 @@
         <v>19</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M14" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="2:16" ht="299.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1717,10 +1717,10 @@
         <v>20</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="2:16" ht="360" customHeight="1" x14ac:dyDescent="0.25">
@@ -1756,10 +1756,10 @@
         <v>20</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1798,7 +1798,7 @@
         <v>131</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1837,7 +1837,7 @@
         <v>131</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1873,10 +1873,10 @@
         <v>19</v>
       </c>
       <c r="L19" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="M19" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="M19" s="10" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="20" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1912,10 +1912,10 @@
         <v>19</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1951,10 +1951,10 @@
         <v>19</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="2:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
@@ -1990,10 +1990,10 @@
         <v>19</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" spans="2:13" ht="268.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -2032,7 +2032,7 @@
         <v>131</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Decision Log v0.10: DEC-011 M15 in E. Lindsay's wording (NotificationSubscriber registered; reportingCounts projection not, OI-14)
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.10.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\decisions\Decision Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EAE6CE6-3AEF-4A84-B50F-33F6FB151391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1824C2AC-5539-4781-A784-5C17199A6FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -497,9 +497,6 @@
     <t>Held; the notification subscriber is registered, the reportingCounts projection is not (TD-001 partly repaid)</t>
   </si>
   <si>
-    <t>The transition service publishes after commit, and the history entry is written inside the transaction, not by a subscriber. At M4 the notification subscriber is registered (src/composition.js, registerSubscribers), so each status change creates an in-application notification for the requester (FR-3.4, Met at the frozen build 6408ab7). The reportingCounts projection is not registered (TD-001 partly repaid): the management view built at M4 counts from requests directly (FR-8.1 to FR-8.6 Met), so the projection and its recovery path (OI-14) are unused. SCP-014 was not admitted.</t>
-  </si>
-  <si>
     <t>Authorisation was designed in, not retrofitted. The route guard is composed once, and a route-table test fails the build if a non-public route lacks it (NFR-3.3). The integration tests caught the wrong-role status (DEF-011), which was fixed in PR #136: a role not permitted for a transition now gets 403 (integration 40 of 40 at 6408ab7). The field-level part, DEC-012 point 3, was not built (OI-16).</t>
   </si>
   <si>
@@ -513,6 +510,9 @@
   </si>
   <si>
     <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream | Version 0.10 (17/10/2026, R. van der Merwe): columns L (Final status, M4) and M (Observed consequence, M4) added for every decision. Columns B to K are unchanged, so each decision reads as it was taken. The cells that waited on the release candidate (DEC-006, DEC-012, DEC-015, DEC-017) were completed on 18/10/2026 from the v4.0-M4-rc evidence, and the DEC-005, DEC-010, DEC-016 and DEC-017 consequences were brought up to date with the CR approvals of 17/10/2026 and the staging runs of 18/10/2026. DEC-016 cites DEF-032; DEC-003 records the staging domain and certificate of 18/10/2026; DEC-015 records the integration job as a required check. After review (18/10/2026): DEC-011 (L15, M15) records the registered notification subscriber, and DEC-004, DEC-013, DEC-018 and DEC-019 (M8, M17, M22, M23) record the M4 fixes and four-browser E2E runs.</t>
+  </si>
+  <si>
+    <t>The transition service publishes after commit, and the history entry is written inside the transaction, not by a subscriber. At M4 the requester-feedback subscriber (NotificationSubscriber, FR-3.4) is registered in the composed application (src/composition.js, PR #136), so a status change reaches the requester as an in-application notification. The reportingCounts projection is not registered, because it has no recovery path (OI-14); the management view counts from requests directly (TD-001 partly repaid, Technical Debt Register v0.4). SCP-014 (delivery by email or push) was not admitted.</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="28" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
@@ -1439,7 +1439,7 @@
         <v>131</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N8" s="20" t="s">
         <v>40</v>
@@ -1720,7 +1720,7 @@
         <v>153</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="2:16" ht="360" customHeight="1" x14ac:dyDescent="0.25">
@@ -1798,7 +1798,7 @@
         <v>131</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1993,7 +1993,7 @@
         <v>139</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="2:13" ht="268.7" customHeight="1" x14ac:dyDescent="0.25">
@@ -2032,7 +2032,7 @@
         <v>131</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>